<commit_message>
Update sample entrant data
</commit_message>
<xml_diff>
--- a/Resultsentrants-aberfeldie-one-hour-track-challenge.xlsx
+++ b/Resultsentrants-aberfeldie-one-hour-track-challenge.xlsx
@@ -5,10 +5,10 @@
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Certificates\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\temp\AthleticsCertificateMaker\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E94180AE-BC43-4CD6-B038-C59B0062E659}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{91DE494F-AD23-46FE-A5D9-F9EF15EB28D1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="22695" windowHeight="14476" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -41,9 +41,6 @@
     <t>Distance</t>
   </si>
   <si>
-    <t>djaus@sportronics.com.au</t>
-  </si>
-  <si>
     <t>Email</t>
   </si>
   <si>
@@ -66,6 +63,9 @@
   </si>
   <si>
     <t>Julie Smith</t>
+  </si>
+  <si>
+    <t>fred@one.com.au</t>
   </si>
 </sst>
 </file>
@@ -450,19 +450,19 @@
   <sheetData>
     <row r="1" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A1" s="3" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B1" t="s">
         <v>0</v>
       </c>
       <c r="C1" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D1" t="s">
         <v>1</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.45">
@@ -470,13 +470,13 @@
         <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C2" s="5" t="s">
-        <v>2</v>
+        <v>10</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E2" s="6"/>
       <c r="I2" s="1"/>
@@ -486,16 +486,16 @@
         <v>2</v>
       </c>
       <c r="B3" t="s">
+        <v>9</v>
+      </c>
+      <c r="C3" s="5" t="s">
         <v>10</v>
-      </c>
-      <c r="C3" s="5" t="s">
-        <v>2</v>
       </c>
       <c r="D3">
         <v>8730</v>
       </c>
       <c r="E3" s="7" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="I3" s="1"/>
     </row>
@@ -504,10 +504,10 @@
         <v>4</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>2</v>
+        <v>10</v>
       </c>
       <c r="D4">
         <v>10145</v>
@@ -560,7 +560,7 @@
   </sheetData>
   <hyperlinks>
     <hyperlink ref="C2" r:id="rId1" xr:uid="{AE62DBFF-6016-41EC-8176-22B76DB75189}"/>
-    <hyperlink ref="C3:C4" r:id="rId2" display="djaus@sportronics.com.au" xr:uid="{818E7673-8737-4ADB-A4C0-15EF568D0229}"/>
+    <hyperlink ref="C3:C4" r:id="rId2" display="fred@one.com.au" xr:uid="{AD3CAEC6-B33E-44C9-B335-88FBE231229D}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>